<commit_message>
Add SDAC Details program (/SdacDetails); confirm CamelHttpPath mapping; p_head char70; update Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DKMFkrrqvWfQdvQXyuumh8
</commit_message>
<xml_diff>
--- a/GeM_CPI_Programs_Inventory.xlsx
+++ b/GeM_CPI_Programs_Inventory.xlsx
@@ -10,7 +10,9 @@
     <sheet name="GeM CPI Programs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Storage &amp; Common Setup" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GeM CPI Programs'!$A$1:$H$12</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -41,12 +43,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
+        <fgColor rgb="001F6391"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00CDEAF6"/>
       </patternFill>
     </fill>
   </fills>
@@ -453,16 +455,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -473,19 +476,19 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Service Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>ABAP Report (Program)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>File Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>API / Service</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>JSON method</t>
@@ -493,10 +496,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CamelHttpPath (URL path default)</t>
+          <t>CamelHttpPath</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Request URL path (p_path)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status / Response handling</t>
         </is>
@@ -510,19 +518,19 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Get Order Summary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>ZGEM_CPI_ORDER_SUMMARY</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_ORDER_SUMMARY.abap</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Order Summary</t>
-        </is>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>orderSummary</t>
@@ -530,10 +538,15 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>/OrderSummary</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>/http/GEM/Sync/OrderSummary</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Done - full typed response (orderIds ALV)</t>
         </is>
@@ -547,19 +560,19 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Get Order Details</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>ZGEM_CPI_ORDER_DETAILS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>ZGEM_CPI_ORDER_DETAILS.abap</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Get Order Details</t>
-        </is>
-      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>getOrders</t>
@@ -567,47 +580,57 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>/OrderDetails</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>/http/GEM/Sync/OrderDetails</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Get Invoice Summary</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_INVOICE_SUMMARY</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_INVOICE_SUMMARY.abap</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Invoice Summary</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>invoiceSummary</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>/InvoiceSummary</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>/http/GEM/Sync/InvoiceSummary</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
@@ -621,19 +644,19 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>Get Invoice Details</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
           <t>ZGEM_CPI_INVOICE_DETAILS</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>ZGEM_CPI_INVOICE_DETAILS.abap</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Invoice Details</t>
-        </is>
-      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>getInvoice</t>
@@ -641,47 +664,57 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
+          <t>/InvoiceDetails</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>/http/GEM/Sync/InvoiceDetails</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>3.6</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Get CRAC Summary</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_CRAC_SUMMARY</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_CRAC_SUMMARY.abap</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>CRAC Summary</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>cracSummary</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>/CracSummary</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>/http/GEM/Sync/CracSummary</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
@@ -695,19 +728,19 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>Get SDAC Summary</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>ZGEM_CPI_SDAC_SUMMARY</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>ZGEM_CPI_SDAC_SUMMARY.abap</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>SDAC Summary</t>
-        </is>
-      </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>cracServiceSummary</t>
@@ -715,47 +748,57 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
+          <t>/SdacSummary</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
           <t>/http/GEM/Sync/SdacSummary</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>3.8</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Get CRAC Details</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_CRAC_DETAILS</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_CRAC_DETAILS.abap</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>CRAC Details</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>getCrac</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>/CracDetails</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>/http/GEM/Sync/CracDetails</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
@@ -764,72 +807,82 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Get SDAC Details</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ZGEM_CPI_SDAC_DETAILS</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>ZGEM_CPI_SDAC_DETAILS.abap</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>getcracservice</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>/SdacDetails</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>/http/GEM/Sync/SdacDetails</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Sample - envelope parsed + raw data</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Get Bill Summary</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_BILL_SUMMARY</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_BILL_SUMMARY.abap</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Bill Summary</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>billSummary</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>/BillSummary</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>/http/GEM/Sync/BillSummary</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Sample - envelope parsed + raw data</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>ZGEM_CPI_BILL_DETAILS</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>ZGEM_CPI_BILL_DETAILS.abap</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Get Bill Details</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>getbills</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>/http/GEM/Sync/BillDetails</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
@@ -838,41 +891,89 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Get Bill Details</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ZGEM_CPI_BILL_DETAILS</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>ZGEM_CPI_BILL_DETAILS.abap</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>getbills</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>/BillDetails</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>/http/GEM/Sync/BillDetails</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Sample - envelope parsed + raw data</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>3.11</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Get Payment Status</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_PAYMENT_STATUS</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>ZGEM_CPI_PAYMENT_STATUS.abap</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Payment Status</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>payments</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>/PaymentStatus</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>/http/GEM/Sync/PaymentStatus</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Sample - envelope parsed + raw data</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -883,11 +984,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -951,88 +1052,112 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Total programs</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>11 (Order Summary + 10 others)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Common - SM59 destination</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>CPI_HTTP_GEM (HTTP type G), Path Prefix EMPTY</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Common - Token</t>
+          <t>Common - SM59 destination</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Proxy ZGEM_TOKENCO_SI_SECURITY_TOKEN (username/password)</t>
+          <t>CPI_HTTP_GEM (HTTP type G), Path Prefix EMPTY</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Common - SEK token header</t>
+          <t>Common - Token</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>token = Bearer &lt;token&gt;</t>
+          <t>Proxy ZGEM_TOKENCO_SI_SECURITY_TOKEN (username/password)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Common - Routing</t>
+          <t>Common - SEK token header</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>URL path -&gt; CPI derives CamelHttpPath (sender endpoint must end with /*)</t>
+          <t>token = Bearer &lt;token&gt;</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Common - Allowed Headers (iFlow)</t>
+          <t>Common - Routing</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>'token' must be whitelisted in sender adapter</t>
+          <t>p_path = /http/GEM/Sync/&lt;Op&gt;  -&gt;  CPI derives CamelHttpPath = /&lt;Op&gt;</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Common - Display</t>
+          <t>Common - iFlow endpoint</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>CL_SALV_TABLE ALV; list header from selection-screen field p_head</t>
+          <t>Sender address must end with /*  (e.g. /GEM/Sync/*)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>Common - Allowed Headers (iFlow)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>'token' must be whitelisted in sender adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Common - Display</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CL_SALV_TABLE ALV; list header from p_head (CHAR70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Skipped - 3.1 Authentication</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Token generation already provided (proxy)</t>
         </is>

</xml_diff>